<commit_message>
Add 14 vision-derived questions from 中国古代文化常识
Coverage: 天文(五星)/历法(太阳神鸟)/乐律(曾侯乙编钟)/职官(令尹·太尉·尚书台)/科举(熹平石经)/礼俗(礼源于祭祀).
Bank now 2043 questions (2000 official + 43 textbook).
</commit_message>
<xml_diff>
--- a/中华文化考研题库_官方+教材补充.xlsx
+++ b/中华文化考研题库_官方+教材补充.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="题库" sheetId="1" r:id="R0cdf055255184f1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="题库" sheetId="1" r:id="Rba5c193281f14aaa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bank" displayName="Bank" ref="A1:L2030" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bank" displayName="Bank" ref="A1:L2044" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="序号"/>
     <x:tableColumn id="2" name="题库"/>
@@ -72463,10 +72463,542 @@
         <x:v>教材命题(视觉识别)</x:v>
       </x:c>
     </x:row>
+    <x:row r="2031">
+      <x:c r="A2031" s="3" t="n">
+        <x:v>2030</x:v>
+      </x:c>
+      <x:c r="B2031" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2031" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2031" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2031" s="3" t="str">
+        <x:v>“五星出东方利中国”织锦护膊出土于新疆民丰县尼雅遗址，其所属历史时期是：</x:v>
+      </x:c>
+      <x:c r="F2031" s="8" t="str">
+        <x:v>西汉</x:v>
+      </x:c>
+      <x:c r="G2031" s="8" t="str">
+        <x:v>东汉</x:v>
+      </x:c>
+      <x:c r="H2031" s="8" t="str">
+        <x:v>汉魏</x:v>
+      </x:c>
+      <x:c r="I2031" s="8" t="str">
+        <x:v>隋唐</x:v>
+      </x:c>
+      <x:c r="J2031" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2031" s="8" t="str">
+        <x:v>该织锦护膊1995年出土于尼雅遗址，教材断代为汉魏时期。</x:v>
+      </x:c>
+      <x:c r="L2031" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2032">
+      <x:c r="A2032" s="3" t="n">
+        <x:v>2031</x:v>
+      </x:c>
+      <x:c r="B2032" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2032" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2032" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2032" s="3" t="str">
+        <x:v>古代天文中的“五星”指的是：</x:v>
+      </x:c>
+      <x:c r="F2032" s="8" t="str">
+        <x:v>金、木、水、火、土五大行星</x:v>
+      </x:c>
+      <x:c r="G2032" s="8" t="str">
+        <x:v>日、月、金、木、水</x:v>
+      </x:c>
+      <x:c r="H2032" s="8" t="str">
+        <x:v>东、南、西、北、中五方星宿</x:v>
+      </x:c>
+      <x:c r="I2032" s="8" t="str">
+        <x:v>紫微、太微、天市三垣及二宿</x:v>
+      </x:c>
+      <x:c r="J2032" s="8" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="K2032" s="8" t="str">
+        <x:v>“五星”即金木水火土五大行星，又称太白、岁星、辰星、荧惑、填星；“五星出东方”指五大行星同现东方天空。</x:v>
+      </x:c>
+      <x:c r="L2032" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2033">
+      <x:c r="A2033" s="3" t="n">
+        <x:v>2032</x:v>
+      </x:c>
+      <x:c r="B2033" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2033" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2033" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2033" s="3" t="str">
+        <x:v>商周时期的“太阳神鸟”金饰出土于哪处遗址？</x:v>
+      </x:c>
+      <x:c r="F2033" s="8" t="str">
+        <x:v>三星堆遗址</x:v>
+      </x:c>
+      <x:c r="G2033" s="8" t="str">
+        <x:v>金沙遗址</x:v>
+      </x:c>
+      <x:c r="H2033" s="8" t="str">
+        <x:v>良渚遗址</x:v>
+      </x:c>
+      <x:c r="I2033" s="8" t="str">
+        <x:v>殷墟遗址</x:v>
+      </x:c>
+      <x:c r="J2033" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2033" s="8" t="str">
+        <x:v>“太阳神鸟”金饰2001年出土于四川成都金沙遗址，属商周时期文物，现为中国文化遗产标志。</x:v>
+      </x:c>
+      <x:c r="L2033" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2034">
+      <x:c r="A2034" s="3" t="n">
+        <x:v>2033</x:v>
+      </x:c>
+      <x:c r="B2034" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2034" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2034" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2034" s="3" t="str">
+        <x:v>曾侯乙编钟1978年出土于湖北随县（今随州），所属时代是：</x:v>
+      </x:c>
+      <x:c r="F2034" s="8" t="str">
+        <x:v>春秋早期</x:v>
+      </x:c>
+      <x:c r="G2034" s="8" t="str">
+        <x:v>战国</x:v>
+      </x:c>
+      <x:c r="H2034" s="8" t="str">
+        <x:v>秦代</x:v>
+      </x:c>
+      <x:c r="I2034" s="8" t="str">
+        <x:v>西汉</x:v>
+      </x:c>
+      <x:c r="J2034" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2034" s="8" t="str">
+        <x:v>曾侯乙编钟1978年出土于湖北随县（今随州市）曾侯乙墓，属战国时期的礼乐重器。</x:v>
+      </x:c>
+      <x:c r="L2034" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2035">
+      <x:c r="A2035" s="3" t="n">
+        <x:v>2034</x:v>
+      </x:c>
+      <x:c r="B2035" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2035" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2035" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2035" s="3" t="str">
+        <x:v>曾侯乙编钟的乐律铭文达三千余字，系统记载音名、阶名、律名，直接证实先秦时期中国已：</x:v>
+      </x:c>
+      <x:c r="F2035" s="8" t="str">
+        <x:v>具备完整的十二半音体系</x:v>
+      </x:c>
+      <x:c r="G2035" s="8" t="str">
+        <x:v>统一度量衡标准</x:v>
+      </x:c>
+      <x:c r="H2035" s="8" t="str">
+        <x:v>发明造纸术</x:v>
+      </x:c>
+      <x:c r="I2035" s="8" t="str">
+        <x:v>掌握铁器冶铸技术</x:v>
+      </x:c>
+      <x:c r="J2035" s="8" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="K2035" s="8" t="str">
+        <x:v>编钟铭文系统记载了音名、阶名、律名，证实战国早期中国已具备完整的十二律（半音）体系。</x:v>
+      </x:c>
+      <x:c r="L2035" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2036">
+      <x:c r="A2036" s="3" t="n">
+        <x:v>2035</x:v>
+      </x:c>
+      <x:c r="B2036" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2036" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2036" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2036" s="3" t="str">
+        <x:v>曾侯乙编钟最具世界性影响的音乐科技成就是：</x:v>
+      </x:c>
+      <x:c r="F2036" s="8" t="str">
+        <x:v>一钟双音，敲击钟体不同部位可发出两个不同音高</x:v>
+      </x:c>
+      <x:c r="G2036" s="8" t="str">
+        <x:v>一钟一音，每钟仅按单一音高铸造</x:v>
+      </x:c>
+      <x:c r="H2036" s="8" t="str">
+        <x:v>钟声浑厚，依托超长共鸣腔实现次声传播</x:v>
+      </x:c>
+      <x:c r="I2036" s="8" t="str">
+        <x:v>钟体镂空，以透雕工艺实现扩音</x:v>
+      </x:c>
+      <x:c r="J2036" s="8" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="K2036" s="8" t="str">
+        <x:v>曾侯乙编钟直观展现“一钟双音”：敲击正鼓部与侧鼓部可获得两个不同音高，突破了传统制钟观念。</x:v>
+      </x:c>
+      <x:c r="L2036" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2037">
+      <x:c r="A2037" s="3" t="n">
+        <x:v>2036</x:v>
+      </x:c>
+      <x:c r="B2037" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2037" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2037" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2037" s="3" t="str">
+        <x:v>战国时期，各国国君之下分设相、将；其中楚国最高长官的称谓是：</x:v>
+      </x:c>
+      <x:c r="F2037" s="8" t="str">
+        <x:v>丞相</x:v>
+      </x:c>
+      <x:c r="G2037" s="8" t="str">
+        <x:v>令尹</x:v>
+      </x:c>
+      <x:c r="H2037" s="8" t="str">
+        <x:v>相国</x:v>
+      </x:c>
+      <x:c r="I2037" s="8" t="str">
+        <x:v>大司马</x:v>
+      </x:c>
+      <x:c r="J2037" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2037" s="8" t="str">
+        <x:v>楚国最高的长官称“令尹”，其下武官最高者为上柱国，与其他各国职官名不同。</x:v>
+      </x:c>
+      <x:c r="L2037" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2038">
+      <x:c r="A2038" s="3" t="n">
+        <x:v>2037</x:v>
+      </x:c>
+      <x:c r="B2038" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2038" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2038" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2038" s="3" t="str">
+        <x:v>秦代中央机构中负责掌管全国军事的官职是：</x:v>
+      </x:c>
+      <x:c r="F2038" s="8" t="str">
+        <x:v>丞相</x:v>
+      </x:c>
+      <x:c r="G2038" s="8" t="str">
+        <x:v>太尉</x:v>
+      </x:c>
+      <x:c r="H2038" s="8" t="str">
+        <x:v>御史大夫</x:v>
+      </x:c>
+      <x:c r="I2038" s="8" t="str">
+        <x:v>大司徒</x:v>
+      </x:c>
+      <x:c r="J2038" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2038" s="8" t="str">
+        <x:v>秦代皇帝之下设丞相（佐理国政）、太尉（掌军事）、御史大夫（掌监察）三府。</x:v>
+      </x:c>
+      <x:c r="L2038" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2039">
+      <x:c r="A2039" s="3" t="n">
+        <x:v>2038</x:v>
+      </x:c>
+      <x:c r="B2039" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2039" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2039" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2039" s="3" t="str">
+        <x:v>东汉光武帝时“虽置三公，事归台阁”，这里的“台阁”实际上成为：</x:v>
+      </x:c>
+      <x:c r="F2039" s="8" t="str">
+        <x:v>最高监察机构</x:v>
+      </x:c>
+      <x:c r="G2039" s="8" t="str">
+        <x:v>外朝执行机构</x:v>
+      </x:c>
+      <x:c r="H2039" s="8" t="str">
+        <x:v>实际的宰相府</x:v>
+      </x:c>
+      <x:c r="I2039" s="8" t="str">
+        <x:v>军事指挥中心</x:v>
+      </x:c>
+      <x:c r="J2039" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2039" s="8" t="str">
+        <x:v>“台阁”指尚书机构；东汉时三公仅处理例行公事，尚书台实掌政务，成为实际上的宰相府。</x:v>
+      </x:c>
+      <x:c r="L2039" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2040">
+      <x:c r="A2040" s="3" t="n">
+        <x:v>2039</x:v>
+      </x:c>
+      <x:c r="B2040" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2040" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2040" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2040" s="3" t="str">
+        <x:v>东汉蔡邕等主持刊刻“熹平石经”的直接背景是：</x:v>
+      </x:c>
+      <x:c r="F2040" s="8" t="str">
+        <x:v>察举制的推行</x:v>
+      </x:c>
+      <x:c r="G2040" s="8" t="str">
+        <x:v>太学经学考试需统一经书文字标准</x:v>
+      </x:c>
+      <x:c r="H2040" s="8" t="str">
+        <x:v>九品中正制的确立</x:v>
+      </x:c>
+      <x:c r="I2040" s="8" t="str">
+        <x:v>科举制的正式形成</x:v>
+      </x:c>
+      <x:c r="J2040" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2040" s="8" t="str">
+        <x:v>熹平石经旨在为太学生和天下儒生提供标准经书文本，与当时太学经学考试、经学定本的需要相关；科举制至隋唐才形成。</x:v>
+      </x:c>
+      <x:c r="L2040" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2041">
+      <x:c r="A2041" s="3" t="n">
+        <x:v>2040</x:v>
+      </x:c>
+      <x:c r="B2041" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2041" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2041" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2041" s="3" t="str">
+        <x:v>东汉《熹平石经》的书体是：</x:v>
+      </x:c>
+      <x:c r="F2041" s="8" t="str">
+        <x:v>小篆</x:v>
+      </x:c>
+      <x:c r="G2041" s="8" t="str">
+        <x:v>隶书（八分书）</x:v>
+      </x:c>
+      <x:c r="H2041" s="8" t="str">
+        <x:v>楷书</x:v>
+      </x:c>
+      <x:c r="I2041" s="8" t="str">
+        <x:v>行书</x:v>
+      </x:c>
+      <x:c r="J2041" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2041" s="8" t="str">
+        <x:v>熹平石经以汉代标准隶书（八分书）书写，字形扁平、波磔分明，与东汉碑刻主流书体一致。</x:v>
+      </x:c>
+      <x:c r="L2041" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2042">
+      <x:c r="A2042" s="3" t="n">
+        <x:v>2041</x:v>
+      </x:c>
+      <x:c r="B2042" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2042" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2042" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2042" s="3" t="str">
+        <x:v>从刊刻目的看，《熹平石经》主要反映了中国古代文化中哪一传统？</x:v>
+      </x:c>
+      <x:c r="F2042" s="8" t="str">
+        <x:v>以法为教、以吏为师</x:v>
+      </x:c>
+      <x:c r="G2042" s="8" t="str">
+        <x:v>民间私学自由讲学</x:v>
+      </x:c>
+      <x:c r="H2042" s="8" t="str">
+        <x:v>经学定本与官方意识形态的规范</x:v>
+      </x:c>
+      <x:c r="I2042" s="8" t="str">
+        <x:v>三教合一的宗教政策</x:v>
+      </x:c>
+      <x:c r="J2042" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2042" s="8" t="str">
+        <x:v>熹平石经是官方校定儒家经书并刻石颁布之举，体现经学定本化与官方借经学统一思想、维护意识形态的传统。</x:v>
+      </x:c>
+      <x:c r="L2042" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2043">
+      <x:c r="A2043" s="3" t="n">
+        <x:v>2042</x:v>
+      </x:c>
+      <x:c r="B2043" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2043" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2043" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2043" s="3" t="str">
+        <x:v>原始社会已出现专用酒器，如陕西宝鸡北首岭出土的仰韶文化“酉瓶”之类器物，最初主要用于：</x:v>
+      </x:c>
+      <x:c r="F2043" s="8" t="str">
+        <x:v>日常饮水</x:v>
+      </x:c>
+      <x:c r="G2043" s="8" t="str">
+        <x:v>祭祀献神</x:v>
+      </x:c>
+      <x:c r="H2043" s="8" t="str">
+        <x:v>储存粮食</x:v>
+      </x:c>
+      <x:c r="I2043" s="8" t="str">
+        <x:v>烹饪食物</x:v>
+      </x:c>
+      <x:c r="J2043" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2043" s="8" t="str">
+        <x:v>礼起源于祭祀；酒在祭祀中用于献神，故酒器与礼俗活动关系密切。</x:v>
+      </x:c>
+      <x:c r="L2043" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2044">
+      <x:c r="A2044" s="3" t="n">
+        <x:v>2043</x:v>
+      </x:c>
+      <x:c r="B2044" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2044" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2044" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2044" s="3" t="str">
+        <x:v>从源流上看，中国古代“礼”的产生与下列哪一活动关系最为密切？</x:v>
+      </x:c>
+      <x:c r="F2044" s="8" t="str">
+        <x:v>农业生产</x:v>
+      </x:c>
+      <x:c r="G2044" s="8" t="str">
+        <x:v>军事战争</x:v>
+      </x:c>
+      <x:c r="H2044" s="8" t="str">
+        <x:v>原始祭祀</x:v>
+      </x:c>
+      <x:c r="I2044" s="8" t="str">
+        <x:v>商业交换</x:v>
+      </x:c>
+      <x:c r="J2044" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2044" s="8" t="str">
+        <x:v>礼俗知识指出礼的源头是原始祭祀活动，祭祀中常以酒器等作为献祭之物，后世礼制由此发展而来。</x:v>
+      </x:c>
+      <x:c r="L2044" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a9afbd49ff64c3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R201b40cc09b541b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
update question bank to 2087
</commit_message>
<xml_diff>
--- a/中华文化考研题库_官方+教材补充.xlsx
+++ b/中华文化考研题库_官方+教材补充.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="题库" sheetId="1" r:id="Rba5c193281f14aaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="题库" sheetId="1" r:id="R0e5a841a8a4c421b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bank" displayName="Bank" ref="A1:L2044" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bank" displayName="Bank" ref="A1:L2088" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="序号"/>
     <x:tableColumn id="2" name="题库"/>
@@ -72995,10 +72995,1682 @@
         <x:v>教材命题(视觉识别)</x:v>
       </x:c>
     </x:row>
+    <x:row r="2045">
+      <x:c r="A2045" s="3" t="n">
+        <x:v>2044</x:v>
+      </x:c>
+      <x:c r="B2045" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2045" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2045" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2045" s="3" t="str">
+        <x:v>下列关于唐代传奇的表述，符合教材所述的是：</x:v>
+      </x:c>
+      <x:c r="F2045" s="8" t="str">
+        <x:v>唐代传奇是封建正史的附庸，以宣扬儒家纲常为主要目的</x:v>
+      </x:c>
+      <x:c r="G2045" s="8" t="str">
+        <x:v>唐代传奇的描写对象从神仙鬼怪转向现实生活，题材扩大到社会各阶层</x:v>
+      </x:c>
+      <x:c r="H2045" s="8" t="str">
+        <x:v>唐代传奇完全继承魏晋志怪小说，专写神仙鬼怪</x:v>
+      </x:c>
+      <x:c r="I2045" s="8" t="str">
+        <x:v>唐代传奇虽具独立文学意识，但缺乏人物与情节</x:v>
+      </x:c>
+      <x:c r="J2045" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2045" s="8" t="str">
+        <x:v>教材指出唐代传奇“不再是封建正史的附庸”，题材转向现实、扩大到文人士子、商贾艺人、豪侠义士、妓女优伶等各阶层。</x:v>
+      </x:c>
+      <x:c r="L2045" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2046">
+      <x:c r="A2046" s="3" t="n">
+        <x:v>2045</x:v>
+      </x:c>
+      <x:c r="B2046" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2046" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2046" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2046" s="3" t="str">
+        <x:v>唐代传奇《柳毅传》的主要情节与主旨是：</x:v>
+      </x:c>
+      <x:c r="F2046" s="8" t="str">
+        <x:v>写洞庭龙君小女受虐待，柳毅传书相救，赞扬救危扶困的品德，具有反封建色彩</x:v>
+      </x:c>
+      <x:c r="G2046" s="8" t="str">
+        <x:v>写文士李益与名妓霍小玉的爱情悲剧</x:v>
+      </x:c>
+      <x:c r="H2046" s="8" t="str">
+        <x:v>写功名富贵如同一梦，带有消极避世思想</x:v>
+      </x:c>
+      <x:c r="I2046" s="8" t="str">
+        <x:v>写虬髯客等豪侠的传奇故事</x:v>
+      </x:c>
+      <x:c r="J2046" s="8" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="K2046" s="8" t="str">
+        <x:v>《柳毅传》写龙女受虐、柳毅传书相救并终成眷属，赞扬其救危扶困品德，寄托对爱情自由的向往。</x:v>
+      </x:c>
+      <x:c r="L2046" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2047">
+      <x:c r="A2047" s="3" t="n">
+        <x:v>2046</x:v>
+      </x:c>
+      <x:c r="B2047" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2047" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2047" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2047" s="3" t="str">
+        <x:v>关于唐代传奇的演变，下列说法正确的是：</x:v>
+      </x:c>
+      <x:c r="F2047" s="8" t="str">
+        <x:v>初唐传奇已完全摆脱志怪痕迹，题材转向现实</x:v>
+      </x:c>
+      <x:c r="G2047" s="8" t="str">
+        <x:v>晚唐多写豪侠故事，《红线》《虬髯客传》为代表作</x:v>
+      </x:c>
+      <x:c r="H2047" s="8" t="str">
+        <x:v>《枕中记》《南柯太守传》是婚姻爱情类代表作</x:v>
+      </x:c>
+      <x:c r="I2047" s="8" t="str">
+        <x:v>《游仙窟》是豪侠故事典范</x:v>
+      </x:c>
+      <x:c r="J2047" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2047" s="8" t="str">
+        <x:v>晚唐传奇多写豪侠，《红线》《虬髯客传》即此类代表；初唐传奇仍带志怪痕迹，《枕中记》《南柯太守传》写功名富贵如梦。</x:v>
+      </x:c>
+      <x:c r="L2047" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2048">
+      <x:c r="A2048" s="3" t="n">
+        <x:v>2047</x:v>
+      </x:c>
+      <x:c r="B2048" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2048" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2048" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2048" s="3" t="str">
+        <x:v>据《尚书》所载，原始人装扮成野兽模仿动作跳舞的早期表演形态被称为：</x:v>
+      </x:c>
+      <x:c r="F2048" s="8" t="str">
+        <x:v>踏摇娘</x:v>
+      </x:c>
+      <x:c r="G2048" s="8" t="str">
+        <x:v>东海黄公</x:v>
+      </x:c>
+      <x:c r="H2048" s="8" t="str">
+        <x:v>百兽率舞</x:v>
+      </x:c>
+      <x:c r="I2048" s="8" t="str">
+        <x:v>优孟衣冠</x:v>
+      </x:c>
+      <x:c r="J2048" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2048" s="8" t="str">
+        <x:v>《尚书》载尧时“百兽率舞”，人装扮野兽模仿其动作，被视为中国戏曲形成的早期萌芽之一。</x:v>
+      </x:c>
+      <x:c r="L2048" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2049">
+      <x:c r="A2049" s="3" t="n">
+        <x:v>2048</x:v>
+      </x:c>
+      <x:c r="B2049" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2049" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2049" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2049" s="3" t="str">
+        <x:v>唐宋流行的“参军戏”中，两个主要角色是：</x:v>
+      </x:c>
+      <x:c r="F2049" s="8" t="str">
+        <x:v>参军、苍鹘</x:v>
+      </x:c>
+      <x:c r="G2049" s="8" t="str">
+        <x:v>副末、副净</x:v>
+      </x:c>
+      <x:c r="H2049" s="8" t="str">
+        <x:v>生、旦</x:v>
+      </x:c>
+      <x:c r="I2049" s="8" t="str">
+        <x:v>末、丑</x:v>
+      </x:c>
+      <x:c r="J2049" s="8" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="K2049" s="8" t="str">
+        <x:v>参军戏有两个固定角色参军与苍鹘，以滑稽调笑、讽刺揶揄为表演特点。</x:v>
+      </x:c>
+      <x:c r="L2049" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2050">
+      <x:c r="A2050" s="3" t="n">
+        <x:v>2049</x:v>
+      </x:c>
+      <x:c r="B2050" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2050" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2050" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2050" s="3" t="str">
+        <x:v>关于宋杂剧与金院本，下列说法正确的是：</x:v>
+      </x:c>
+      <x:c r="F2050" s="8" t="str">
+        <x:v>二者均有完整剧本流传至今</x:v>
+      </x:c>
+      <x:c r="G2050" s="8" t="str">
+        <x:v>宋杂剧在参军戏基础上发展，角色由两个增至五个</x:v>
+      </x:c>
+      <x:c r="H2050" s="8" t="str">
+        <x:v>二者尚不具备戏曲雏形</x:v>
+      </x:c>
+      <x:c r="I2050" s="8" t="str">
+        <x:v>元杂剧并非在其基础上发展而来</x:v>
+      </x:c>
+      <x:c r="J2050" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2050" s="8" t="str">
+        <x:v>宋杂剧在参军戏基础上发展，角色由参军、苍鹘两个增至五个，金院本与之相似，均已具戏曲雏形，元杂剧由此发展而来。</x:v>
+      </x:c>
+      <x:c r="L2050" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2051">
+      <x:c r="A2051" s="3" t="n">
+        <x:v>2050</x:v>
+      </x:c>
+      <x:c r="B2051" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2051" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2051" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2051" s="3" t="str">
+        <x:v>据《汉书·律历志》，古代“黄钟”在度量衡标准中的特殊作用是：</x:v>
+      </x:c>
+      <x:c r="F2051" s="8" t="str">
+        <x:v>仅作乐器定音的标准</x:v>
+      </x:c>
+      <x:c r="G2051" s="8" t="str">
+        <x:v>是确立长度、容积、重量的共同基础</x:v>
+      </x:c>
+      <x:c r="H2051" s="8" t="str">
+        <x:v>专用于测量土地面积</x:v>
+      </x:c>
+      <x:c r="I2051" s="8" t="str">
+        <x:v>汉代以后才规定的标准</x:v>
+      </x:c>
+      <x:c r="J2051" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2051" s="8" t="str">
+        <x:v>古人以黄钟律管的长、容积及所容黍重分别确定度（长度）、量（容积）、权衡（重量）标准。</x:v>
+      </x:c>
+      <x:c r="L2051" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2052">
+      <x:c r="A2052" s="3" t="n">
+        <x:v>2051</x:v>
+      </x:c>
+      <x:c r="B2052" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2052" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2052" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2052" s="3" t="str">
+        <x:v>按照《汉书·律历志》记载的权衡进位，一两等于多少铢？</x:v>
+      </x:c>
+      <x:c r="F2052" s="8" t="str">
+        <x:v>十铢</x:v>
+      </x:c>
+      <x:c r="G2052" s="8" t="str">
+        <x:v>十二铢</x:v>
+      </x:c>
+      <x:c r="H2052" s="8" t="str">
+        <x:v>二十四铢</x:v>
+      </x:c>
+      <x:c r="I2052" s="8" t="str">
+        <x:v>八铢</x:v>
+      </x:c>
+      <x:c r="J2052" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2052" s="8" t="str">
+        <x:v>原文：“二十四铢为两，十六两为斤，三十斤为钧，四钧为石。”</x:v>
+      </x:c>
+      <x:c r="L2052" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2053">
+      <x:c r="A2053" s="3" t="n">
+        <x:v>2052</x:v>
+      </x:c>
+      <x:c r="B2053" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2053" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2053" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2053" s="3" t="str">
+        <x:v>《百家姓》以“赵钱孙李”开头，主要是因为：</x:v>
+      </x:c>
+      <x:c r="F2053" s="8" t="str">
+        <x:v>按姓氏人口多少排序</x:v>
+      </x:c>
+      <x:c r="G2053" s="8" t="str">
+        <x:v>按姓氏产生先后排序</x:v>
+      </x:c>
+      <x:c r="H2053" s="8" t="str">
+        <x:v>北宋以“赵”为国姓，其余多为当朝望族</x:v>
+      </x:c>
+      <x:c r="I2053" s="8" t="str">
+        <x:v>清代官方颁布的姓氏等级</x:v>
+      </x:c>
+      <x:c r="J2053" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2053" s="8" t="str">
+        <x:v>《百家姓》成书于北宋初，以宋国姓“赵”居首，其余多为望族大姓，反映政治权势对姓氏排序的影响。</x:v>
+      </x:c>
+      <x:c r="L2053" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2054">
+      <x:c r="A2054" s="3" t="n">
+        <x:v>2053</x:v>
+      </x:c>
+      <x:c r="B2054" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2054" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2054" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2054" s="3" t="str">
+        <x:v>《百家姓》的部分版本将“朱”姓置于前列，主要原因是：</x:v>
+      </x:c>
+      <x:c r="F2054" s="8" t="str">
+        <x:v>朱姓当时人口最多</x:v>
+      </x:c>
+      <x:c r="G2054" s="8" t="str">
+        <x:v>编著者姓朱</x:v>
+      </x:c>
+      <x:c r="H2054" s="8" t="str">
+        <x:v>宋代皇室姓赵而朱为唐代望族</x:v>
+      </x:c>
+      <x:c r="I2054" s="8" t="str">
+        <x:v>明代皇室姓朱，版本在明代流传中被提前以尊当朝</x:v>
+      </x:c>
+      <x:c r="J2054" s="8" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="K2054" s="8" t="str">
+        <x:v>《百家姓》成书于北宋，明代大量刊刻流传，因明帝姓朱，部分版本把“朱”姓提前以示尊崇当朝皇权。</x:v>
+      </x:c>
+      <x:c r="L2054" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2055">
+      <x:c r="A2055" s="3" t="n">
+        <x:v>2054</x:v>
+      </x:c>
+      <x:c r="B2055" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2055" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2055" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2055" s="3" t="str">
+        <x:v>关于中国古代宗法制度，下列表述正确的是：</x:v>
+      </x:c>
+      <x:c r="F2055" s="8" t="str">
+        <x:v>核心是嫡长子继承制，旨在维护贵族内部等级秩序</x:v>
+      </x:c>
+      <x:c r="G2055" s="8" t="str">
+        <x:v>大宗与小宗是绝对平等的政治关系</x:v>
+      </x:c>
+      <x:c r="H2055" s="8" t="str">
+        <x:v>仅适用于皇室，与民间宗族无关</x:v>
+      </x:c>
+      <x:c r="I2055" s="8" t="str">
+        <x:v>西周形成后至秦汉已彻底消亡</x:v>
+      </x:c>
+      <x:c r="J2055" s="8" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="K2055" s="8" t="str">
+        <x:v>宗法以嫡长子继承为核心，通过大宗、小宗区分维护等级秩序；其影响及于民间宗族并延续后世。</x:v>
+      </x:c>
+      <x:c r="L2055" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2056">
+      <x:c r="A2056" s="3" t="n">
+        <x:v>2055</x:v>
+      </x:c>
+      <x:c r="B2056" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2056" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2056" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2056" s="3" t="str">
+        <x:v>关于宗族“宗祠”的作用，下列符合史实的是：</x:v>
+      </x:c>
+      <x:c r="F2056" s="8" t="str">
+        <x:v>祭祀祖先、处理宗族事务的重要场所</x:v>
+      </x:c>
+      <x:c r="G2056" s="8" t="str">
+        <x:v>由官府统一规划并直接管理</x:v>
+      </x:c>
+      <x:c r="H2056" s="8" t="str">
+        <x:v>严禁举行任何家族聚会</x:v>
+      </x:c>
+      <x:c r="I2056" s="8" t="str">
+        <x:v>唐代以后才出现，此前无类似建筑</x:v>
+      </x:c>
+      <x:c r="J2056" s="8" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="K2056" s="8" t="str">
+        <x:v>宗祠是宗族祭祀祖先、议事与管理族产的场所，由宗族自行修建管理；家庙宗祠形态先秦已有雏形。</x:v>
+      </x:c>
+      <x:c r="L2056" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2057">
+      <x:c r="A2057" s="3" t="n">
+        <x:v>2056</x:v>
+      </x:c>
+      <x:c r="B2057" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2057" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2057" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2057" s="3" t="str">
+        <x:v>宗法制度下“大宗”与“小宗”的关系是：</x:v>
+      </x:c>
+      <x:c r="F2057" s="8" t="str">
+        <x:v>小宗须服从大宗，具有相对隶属关系</x:v>
+      </x:c>
+      <x:c r="G2057" s="8" t="str">
+        <x:v>二者在血缘上毫无关联</x:v>
+      </x:c>
+      <x:c r="H2057" s="8" t="str">
+        <x:v>小宗在宗族事务中拥有更高决策权</x:v>
+      </x:c>
+      <x:c r="I2057" s="8" t="str">
+        <x:v>仅以年龄大小区分，与血缘传承无关</x:v>
+      </x:c>
+      <x:c r="J2057" s="8" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="K2057" s="8" t="str">
+        <x:v>大宗为宗族最高代表，小宗须服从大宗；二者有血缘关联，区分依据是嫡庶继承关系而非年龄。</x:v>
+      </x:c>
+      <x:c r="L2057" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2058">
+      <x:c r="A2058" s="3" t="n">
+        <x:v>2057</x:v>
+      </x:c>
+      <x:c r="B2058" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2058" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2058" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2058" s="3" t="str">
+        <x:v>汉代陶质明器仓廪上书有“稻米”“黍”“粟”“万石”等字样，主要反映的是：</x:v>
+      </x:c>
+      <x:c r="F2058" s="8" t="str">
+        <x:v>服饰等级观念</x:v>
+      </x:c>
+      <x:c r="G2058" s="8" t="str">
+        <x:v>农业仓储与祈求丰收的观念</x:v>
+      </x:c>
+      <x:c r="H2058" s="8" t="str">
+        <x:v>居住建筑形制</x:v>
+      </x:c>
+      <x:c r="I2058" s="8" t="str">
+        <x:v>车马出行制度</x:v>
+      </x:c>
+      <x:c r="J2058" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2058" s="8" t="str">
+        <x:v>明器陶仓盛放谷物之模型，上书粮名与“万石”寓意仓廪充实，反映汉代人祈望农业丰收、储粮充足的心理。</x:v>
+      </x:c>
+      <x:c r="L2058" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2059">
+      <x:c r="A2059" s="3" t="n">
+        <x:v>2058</x:v>
+      </x:c>
+      <x:c r="B2059" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2059" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2059" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2059" s="3" t="str">
+        <x:v>魏晋南北朝时期，随着儒学独尊地位动摇，一种融合儒道哲理、探讨“有无本末”的哲学思潮兴起，它是：</x:v>
+      </x:c>
+      <x:c r="F2059" s="8" t="str">
+        <x:v>程朱理学</x:v>
+      </x:c>
+      <x:c r="G2059" s="8" t="str">
+        <x:v>魏晋玄学</x:v>
+      </x:c>
+      <x:c r="H2059" s="8" t="str">
+        <x:v>阳明心学</x:v>
+      </x:c>
+      <x:c r="I2059" s="8" t="str">
+        <x:v>乾嘉朴学</x:v>
+      </x:c>
+      <x:c r="J2059" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2059" s="8" t="str">
+        <x:v>魏晋玄学是儒家与道家思想在哲理层面的融合，以“有无本末”为核心议题。</x:v>
+      </x:c>
+      <x:c r="L2059" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2060">
+      <x:c r="A2060" s="3" t="n">
+        <x:v>2059</x:v>
+      </x:c>
+      <x:c r="B2060" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2060" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2060" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2060" s="3" t="str">
+        <x:v>关于魏晋玄学代表王弼“以无为本”的思想，下列说法符合教材的是：</x:v>
+      </x:c>
+      <x:c r="F2060" s="8" t="str">
+        <x:v>“无”是某种具体有形之物</x:v>
+      </x:c>
+      <x:c r="G2060" s="8" t="str">
+        <x:v>“无”是无形无名、不具任何规定性的万物之本</x:v>
+      </x:c>
+      <x:c r="H2060" s="8" t="str">
+        <x:v>“无”仅指空间上的空无</x:v>
+      </x:c>
+      <x:c r="I2060" s="8" t="str">
+        <x:v>王弼主张“言尽意”，语言可完全表达玄理</x:v>
+      </x:c>
+      <x:c r="J2060" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2060" s="8" t="str">
+        <x:v>王弼认为“无”无形无名、超言绝象、不具规定性，是万物之宗（以无为本）。</x:v>
+      </x:c>
+      <x:c r="L2060" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2061">
+      <x:c r="A2061" s="3" t="n">
+        <x:v>2060</x:v>
+      </x:c>
+      <x:c r="B2061" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2061" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2061" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2061" s="3" t="str">
+        <x:v>下列选项中，不属于魏晋玄学辩论核心议题的是：</x:v>
+      </x:c>
+      <x:c r="F2061" s="8" t="str">
+        <x:v>有无本末</x:v>
+      </x:c>
+      <x:c r="G2061" s="8" t="str">
+        <x:v>言不尽意</x:v>
+      </x:c>
+      <x:c r="H2061" s="8" t="str">
+        <x:v>格物致知</x:v>
+      </x:c>
+      <x:c r="I2061" s="8" t="str">
+        <x:v>声无哀乐</x:v>
+      </x:c>
+      <x:c r="J2061" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2061" s="8" t="str">
+        <x:v>玄学议题包括有无本末、言不尽意、声无哀乐、才性四本等；“格物致知”属后世宋明理学。</x:v>
+      </x:c>
+      <x:c r="L2061" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2062">
+      <x:c r="A2062" s="3" t="n">
+        <x:v>2061</x:v>
+      </x:c>
+      <x:c r="B2062" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2062" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2062" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2062" s="3" t="str">
+        <x:v>朱熹主张“理在气先”又言“理未尝离乎气”，其“理在气先”的含义是：</x:v>
+      </x:c>
+      <x:c r="F2062" s="8" t="str">
+        <x:v>理在时间上先于气产生</x:v>
+      </x:c>
+      <x:c r="G2062" s="8" t="str">
+        <x:v>理是逻辑上在先的本原，气是具体生成的材质</x:v>
+      </x:c>
+      <x:c r="H2062" s="8" t="str">
+        <x:v>气是第一性，理依附于气</x:v>
+      </x:c>
+      <x:c r="I2062" s="8" t="str">
+        <x:v>理与气是各自独立的两种实体</x:v>
+      </x:c>
+      <x:c r="J2062" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2062" s="8" t="str">
+        <x:v>朱熹以理为形而上之本、气为形而下之器，“理在气先”指逻辑上的本末关系而非时间先后。</x:v>
+      </x:c>
+      <x:c r="L2062" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2063">
+      <x:c r="A2063" s="3" t="n">
+        <x:v>2062</x:v>
+      </x:c>
+      <x:c r="B2063" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2063" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2063" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2063" s="3" t="str">
+        <x:v>朱熹提出“理一分殊”，并以“月印万川”比喻，意在说明：</x:v>
+      </x:c>
+      <x:c r="F2063" s="8" t="str">
+        <x:v>万物各有完全独立的理，互不相关</x:v>
+      </x:c>
+      <x:c r="G2063" s="8" t="str">
+        <x:v>物质世界（气）是万物产生的根本</x:v>
+      </x:c>
+      <x:c r="H2063" s="8" t="str">
+        <x:v>天地间有一个总的“太极”之理，万物分禀此理而存在</x:v>
+      </x:c>
+      <x:c r="I2063" s="8" t="str">
+        <x:v>“理一分殊”与佛教学说完全等同</x:v>
+      </x:c>
+      <x:c r="J2063" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2063" s="8" t="str">
+        <x:v>“理一分殊”谓太极即理一，万物之理皆出于此而各有分殊，如月印万川而月唯一。</x:v>
+      </x:c>
+      <x:c r="L2063" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2064">
+      <x:c r="A2064" s="3" t="n">
+        <x:v>2063</x:v>
+      </x:c>
+      <x:c r="B2064" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2064" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2064" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2064" s="3" t="str">
+        <x:v>朱熹在人性论上区分“道心”与“人心”，其观点是：</x:v>
+      </x:c>
+      <x:c r="F2064" s="8" t="str">
+        <x:v>道心指常人的气质，人心指圣贤之性</x:v>
+      </x:c>
+      <x:c r="G2064" s="8" t="str">
+        <x:v>人性本恶，须“灭人欲”才能向善</x:v>
+      </x:c>
+      <x:c r="H2064" s="8" t="str">
+        <x:v>道心出于天理，人心出于形气之私，须以天理节制人欲</x:v>
+      </x:c>
+      <x:c r="I2064" s="8" t="str">
+        <x:v>“存天理灭人欲”旨在压制百姓基本生存需求</x:v>
+      </x:c>
+      <x:c r="J2064" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2064" s="8" t="str">
+        <x:v>朱熹谓道心为纯然天理、人心为形气之私，主张以修养存天理、灭人欲，使道德理性支配欲望。</x:v>
+      </x:c>
+      <x:c r="L2064" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2065">
+      <x:c r="A2065" s="3" t="n">
+        <x:v>2064</x:v>
+      </x:c>
+      <x:c r="B2065" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2065" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2065" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2065" s="3" t="str">
+        <x:v>关于古代“简牍”，下列说法正确的是：</x:v>
+      </x:c>
+      <x:c r="F2065" s="8" t="str">
+        <x:v>简牍为纸普及前的主要书写材料，最早出现于汉代</x:v>
+      </x:c>
+      <x:c r="G2065" s="8" t="str">
+        <x:v>现存最早竹简出自曾侯乙墓，证明商代已用简牍</x:v>
+      </x:c>
+      <x:c r="H2065" s="8" t="str">
+        <x:v>简宽一般有 1 厘米与 2 厘米两种，宽 1 厘米者通常只抄一行字</x:v>
+      </x:c>
+      <x:c r="I2065" s="8" t="str">
+        <x:v>简牍通行于商代至秦汉，造纸术普及后被彻底取代</x:v>
+      </x:c>
+      <x:c r="J2065" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2065" s="8" t="str">
+        <x:v>简的宽度约分 1 厘米与 2 厘米两种，窄者只抄一行字；最早简属战国早期，简牍通行期自东周至魏晋。</x:v>
+      </x:c>
+      <x:c r="L2065" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2066">
+      <x:c r="A2066" s="3" t="n">
+        <x:v>2065</x:v>
+      </x:c>
+      <x:c r="B2066" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2066" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2066" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2066" s="3" t="str">
+        <x:v>关于古代简牍的形制与称谓，下列说法不正确的是：</x:v>
+      </x:c>
+      <x:c r="F2066" s="8" t="str">
+        <x:v>写诏书的简长一尺一寸，称“尺一之诏”</x:v>
+      </x:c>
+      <x:c r="G2066" s="8" t="str">
+        <x:v>写经传的简长可达汉尺二尺四寸</x:v>
+      </x:c>
+      <x:c r="H2066" s="8" t="str">
+        <x:v>三尺长的简写律令，故有“三尺法”之说</x:v>
+      </x:c>
+      <x:c r="I2066" s="8" t="str">
+        <x:v>一尺长的牍多用于写信，后世遂以“尺牍”称书信</x:v>
+      </x:c>
+      <x:c r="J2066" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2066" s="8" t="str">
+        <x:v>写儒家经典的简长二尺四寸，写经传之简稍短（二尺一寸左右），B 将经传误为二尺四寸。</x:v>
+      </x:c>
+      <x:c r="L2066" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2067">
+      <x:c r="A2067" s="3" t="n">
+        <x:v>2066</x:v>
+      </x:c>
+      <x:c r="B2067" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2067" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2067" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2067" s="3" t="str">
+        <x:v>从营造起源看，早期人类选择洞穴、河岸等栖息地，最初的功能诉求是：</x:v>
+      </x:c>
+      <x:c r="F2067" s="8" t="str">
+        <x:v>彰显权力与等级</x:v>
+      </x:c>
+      <x:c r="G2067" s="8" t="str">
+        <x:v>抵御自然侵袭、获得生存庇护</x:v>
+      </x:c>
+      <x:c r="H2067" s="8" t="str">
+        <x:v>满足祭祀礼仪需要</x:v>
+      </x:c>
+      <x:c r="I2067" s="8" t="str">
+        <x:v>追求审美装饰效果</x:v>
+      </x:c>
+      <x:c r="J2067" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2067" s="8" t="str">
+        <x:v>宫室建筑源于人类求生存安全的基本需求（避风雨野兽、就近水源），礼制、祭祀、审美是后起功能。</x:v>
+      </x:c>
+      <x:c r="L2067" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2068">
+      <x:c r="A2068" s="3" t="n">
+        <x:v>2067</x:v>
+      </x:c>
+      <x:c r="B2068" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2068" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2068" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2068" s="3" t="str">
+        <x:v>依先秦车马礼制“天子驾六”之制，天、诸侯、大夫各自驾马数为：</x:v>
+      </x:c>
+      <x:c r="F2068" s="8" t="str">
+        <x:v>天子六、诸侯五、大夫四</x:v>
+      </x:c>
+      <x:c r="G2068" s="8" t="str">
+        <x:v>天子六、诸侯四、大夫二</x:v>
+      </x:c>
+      <x:c r="H2068" s="8" t="str">
+        <x:v>天子四、诸侯三、大夫二</x:v>
+      </x:c>
+      <x:c r="I2068" s="8" t="str">
+        <x:v>天子六、诸侯六、大夫四</x:v>
+      </x:c>
+      <x:c r="J2068" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2068" s="8" t="str">
+        <x:v>“天子驾六”即天子驾六马、诸侯驾四、大夫驾二，出土的东周天子驾六车马坑为其实证。</x:v>
+      </x:c>
+      <x:c r="L2068" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2069">
+      <x:c r="A2069" s="3" t="n">
+        <x:v>2068</x:v>
+      </x:c>
+      <x:c r="B2069" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2069" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2069" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2069" s="3" t="str">
+        <x:v>河南洛阳出土的东周“天子驾六”车马坑，其文化意义主要在于：</x:v>
+      </x:c>
+      <x:c r="F2069" s="8" t="str">
+        <x:v>证明东周已普遍使用六马驾车</x:v>
+      </x:c>
+      <x:c r="G2069" s="8" t="str">
+        <x:v>印证古文献中“天子驾六”礼制的记载</x:v>
+      </x:c>
+      <x:c r="H2069" s="8" t="str">
+        <x:v>表明车马葬制已取代人殉</x:v>
+      </x:c>
+      <x:c r="I2069" s="8" t="str">
+        <x:v>说明洛阳为东周唯一政治中心</x:v>
+      </x:c>
+      <x:c r="J2069" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2069" s="8" t="str">
+        <x:v>该车马坑为“天子驾六”提供实物证据，与文献记载相互印证，而非普遍使用或取代人殉等。</x:v>
+      </x:c>
+      <x:c r="L2069" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2070">
+      <x:c r="A2070" s="3" t="n">
+        <x:v>2069</x:v>
+      </x:c>
+      <x:c r="B2070" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2070" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2070" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2070" s="3" t="str">
+        <x:v>关于古代车马与礼制的关系，下列说法正确的是：</x:v>
+      </x:c>
+      <x:c r="F2070" s="8" t="str">
+        <x:v>车马多少仅代表财富，与等级无关</x:v>
+      </x:c>
+      <x:c r="G2070" s="8" t="str">
+        <x:v>车马是身份地位象征，使用规格有严格等级规定</x:v>
+      </x:c>
+      <x:c r="H2070" s="8" t="str">
+        <x:v>东周已废除车马随葬制度</x:v>
+      </x:c>
+      <x:c r="I2070" s="8" t="str">
+        <x:v>只有天子可用马车，诸侯以下一律禁止乘车</x:v>
+      </x:c>
+      <x:c r="J2070" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2070" s="8" t="str">
+        <x:v>车马既是交通工具更是礼制载体，不同等级对应不同规格（如天子驾六），诸侯以下可用但规格受限。</x:v>
+      </x:c>
+      <x:c r="L2070" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2071">
+      <x:c r="A2071" s="3" t="n">
+        <x:v>2070</x:v>
+      </x:c>
+      <x:c r="B2071" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2071" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2071" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2071" s="3" t="str">
+        <x:v>古代帝王礼服上的“十二章”纹样（日、月、星辰、山、龙、华虫等），主要象征：</x:v>
+      </x:c>
+      <x:c r="F2071" s="8" t="str">
+        <x:v>皇帝个人的艺术审美</x:v>
+      </x:c>
+      <x:c r="G2071" s="8" t="str">
+        <x:v>皇权至高无上与帝德规范</x:v>
+      </x:c>
+      <x:c r="H2071" s="8" t="str">
+        <x:v>满族特有的骑射文化</x:v>
+      </x:c>
+      <x:c r="I2071" s="8" t="str">
+        <x:v>服饰的实用保暖功能</x:v>
+      </x:c>
+      <x:c r="J2071" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2071" s="8" t="str">
+        <x:v>十二章纹是帝王礼服传统纹样，各纹有象征意义，整体体现皇权天授与帝王品德规范。</x:v>
+      </x:c>
+      <x:c r="L2071" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2072">
+      <x:c r="A2072" s="3" t="n">
+        <x:v>2071</x:v>
+      </x:c>
+      <x:c r="B2072" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2072" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2072" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2072" s="3" t="str">
+        <x:v>宋代文学高度繁荣，其标志性文学体裁是：</x:v>
+      </x:c>
+      <x:c r="F2072" s="8" t="str">
+        <x:v>诗</x:v>
+      </x:c>
+      <x:c r="G2072" s="8" t="str">
+        <x:v>词</x:v>
+      </x:c>
+      <x:c r="H2072" s="8" t="str">
+        <x:v>曲</x:v>
+      </x:c>
+      <x:c r="I2072" s="8" t="str">
+        <x:v>赋</x:v>
+      </x:c>
+      <x:c r="J2072" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2072" s="8" t="str">
+        <x:v>宋代是词高度繁荣的时期，词成为宋代文学的标志性体裁。</x:v>
+      </x:c>
+      <x:c r="L2072" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2073">
+      <x:c r="A2073" s="3" t="n">
+        <x:v>2072</x:v>
+      </x:c>
+      <x:c r="B2073" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2073" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2073" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2073" s="3" t="str">
+        <x:v>宋初词坛主要继承晚唐五代的婉丽风气，其代表性词人是：</x:v>
+      </x:c>
+      <x:c r="F2073" s="8" t="str">
+        <x:v>苏轼、辛弃疾</x:v>
+      </x:c>
+      <x:c r="G2073" s="8" t="str">
+        <x:v>晏殊、晏几道</x:v>
+      </x:c>
+      <x:c r="H2073" s="8" t="str">
+        <x:v>周邦彦、姜夔</x:v>
+      </x:c>
+      <x:c r="I2073" s="8" t="str">
+        <x:v>张炎、王沂孙</x:v>
+      </x:c>
+      <x:c r="J2073" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2073" s="8" t="str">
+        <x:v>宋初词坛承晚唐五代婉丽之风，晏殊、晏几道父子为代表性词人；豪放派至苏轼、辛弃疾而兴。</x:v>
+      </x:c>
+      <x:c r="L2073" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2074">
+      <x:c r="A2074" s="3" t="n">
+        <x:v>2073</x:v>
+      </x:c>
+      <x:c r="B2074" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2074" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2074" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2074" s="3" t="str">
+        <x:v>较早以《渔家傲》把边塞风云引入词坛、开开阔深沉意境的词人是：</x:v>
+      </x:c>
+      <x:c r="F2074" s="8" t="str">
+        <x:v>晏殊</x:v>
+      </x:c>
+      <x:c r="G2074" s="8" t="str">
+        <x:v>欧阳修</x:v>
+      </x:c>
+      <x:c r="H2074" s="8" t="str">
+        <x:v>范仲淹</x:v>
+      </x:c>
+      <x:c r="I2074" s="8" t="str">
+        <x:v>晏几道</x:v>
+      </x:c>
+      <x:c r="J2074" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2074" s="8" t="str">
+        <x:v>范仲淹《渔家傲·秋思》抒边防将士忧国情怀，将边塞题材引入词中，意境开阔深沉。</x:v>
+      </x:c>
+      <x:c r="L2074" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2075">
+      <x:c r="A2075" s="3" t="n">
+        <x:v>2074</x:v>
+      </x:c>
+      <x:c r="B2075" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2075" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2075" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2075" s="3" t="str">
+        <x:v>明代陈献章论学“以自然为宗”，其修养工夫主张是：</x:v>
+      </x:c>
+      <x:c r="F2075" s="8" t="str">
+        <x:v>天地万物皆吾心之产物</x:v>
+      </x:c>
+      <x:c r="G2075" s="8" t="str">
+        <x:v>为学须在事物上求理</x:v>
+      </x:c>
+      <x:c r="H2075" s="8" t="str">
+        <x:v>静坐中养出端倪</x:v>
+      </x:c>
+      <x:c r="I2075" s="8" t="str">
+        <x:v>知先行后、以知为后</x:v>
+      </x:c>
+      <x:c r="J2075" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2075" s="8" t="str">
+        <x:v>陈献章主张“静坐中养出端倪”，强调内心体认，是理学向心学转向的重要环节。</x:v>
+      </x:c>
+      <x:c r="L2075" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2076">
+      <x:c r="A2076" s="3" t="n">
+        <x:v>2075</x:v>
+      </x:c>
+      <x:c r="B2076" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2076" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2076" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2076" s="3" t="str">
+        <x:v>王守仁“致良知”学说在修养工夫上强调：</x:v>
+      </x:c>
+      <x:c r="F2076" s="8" t="str">
+        <x:v>格物穷理、即物求理</x:v>
+      </x:c>
+      <x:c r="G2076" s="8" t="str">
+        <x:v>事上磨练、知行合一</x:v>
+      </x:c>
+      <x:c r="H2076" s="8" t="str">
+        <x:v>静坐澄心、一循天理</x:v>
+      </x:c>
+      <x:c r="I2076" s="8" t="str">
+        <x:v>读书穷理、问学辨思</x:v>
+      </x:c>
+      <x:c r="J2076" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2076" s="8" t="str">
+        <x:v>王守仁心学主张知行合一、致良知，工夫重在“事上磨练”，与向外求理的程朱路向不同。</x:v>
+      </x:c>
+      <x:c r="L2076" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2077">
+      <x:c r="A2077" s="3" t="n">
+        <x:v>2076</x:v>
+      </x:c>
+      <x:c r="B2077" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2077" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2077" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2077" s="3" t="str">
+        <x:v>关于雕版印刷术的发明年代，下列说法正确的是：</x:v>
+      </x:c>
+      <x:c r="F2077" s="8" t="str">
+        <x:v>唐代文献可确证其发明于唐代</x:v>
+      </x:c>
+      <x:c r="G2077" s="8" t="str">
+        <x:v>据韩国发现的《陀罗尼经》应发明于韩国</x:v>
+      </x:c>
+      <x:c r="H2077" s="8" t="str">
+        <x:v>目前虽无确切年代，但至迟在唐代已出现应用</x:v>
+      </x:c>
+      <x:c r="I2077" s="8" t="str">
+        <x:v>雕版印刷发明于宋代，早于活字印刷</x:v>
+      </x:c>
+      <x:c r="J2077" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2077" s="8" t="str">
+        <x:v>雕版印刷确切发明年代尚难确定，但七世纪中叶已出现、至迟唐代已应用；1966 年发现的最早印刷品被认为是唐印本。</x:v>
+      </x:c>
+      <x:c r="L2077" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2078">
+      <x:c r="A2078" s="3" t="n">
+        <x:v>2077</x:v>
+      </x:c>
+      <x:c r="B2078" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2078" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2078" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2078" s="3" t="str">
+        <x:v>与雕版印刷相比，下列不属于活字印刷优势的是：</x:v>
+      </x:c>
+      <x:c r="F2078" s="8" t="str">
+        <x:v>印刷效率高，可大量印制</x:v>
+      </x:c>
+      <x:c r="G2078" s="8" t="str">
+        <x:v>活字可反复使用，节省费用</x:v>
+      </x:c>
+      <x:c r="H2078" s="8" t="str">
+        <x:v>无需制字刻版，省去排版工序</x:v>
+      </x:c>
+      <x:c r="I2078" s="8" t="str">
+        <x:v>排版灵活，遇缺字可随时补刻</x:v>
+      </x:c>
+      <x:c r="J2078" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2078" s="8" t="str">
+        <x:v>活字印刷仍须先制作单个活字再排版，并非“无需刻版”，故 C 不属于其优势。</x:v>
+      </x:c>
+      <x:c r="L2078" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2079">
+      <x:c r="A2079" s="3" t="n">
+        <x:v>2078</x:v>
+      </x:c>
+      <x:c r="B2079" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2079" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2079" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2079" s="3" t="str">
+        <x:v>据教材，印刷术发明所必需的技术基础是：</x:v>
+      </x:c>
+      <x:c r="F2079" s="8" t="str">
+        <x:v>松烟墨的普遍使用</x:v>
+      </x:c>
+      <x:c r="G2079" s="8" t="str">
+        <x:v>掌握反文印刷原理与刻字技术</x:v>
+      </x:c>
+      <x:c r="H2079" s="8" t="str">
+        <x:v>纸张的普及与广泛应用</x:v>
+      </x:c>
+      <x:c r="I2079" s="8" t="str">
+        <x:v>彩色套印技术的出现</x:v>
+      </x:c>
+      <x:c r="J2079" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2079" s="8" t="str">
+        <x:v>印刷术除纸、墨等物质条件外，还须掌握刻字工艺与“反文印刷”原理，后者即技术基础。</x:v>
+      </x:c>
+      <x:c r="L2079" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2080">
+      <x:c r="A2080" s="3" t="n">
+        <x:v>2079</x:v>
+      </x:c>
+      <x:c r="B2080" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2080" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2080" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2080" s="3" t="str">
+        <x:v>据教材，商周以前人们对一年季节的认识是：</x:v>
+      </x:c>
+      <x:c r="F2080" s="8" t="str">
+        <x:v>一年只分春秋二时，春秋可代表一年</x:v>
+      </x:c>
+      <x:c r="G2080" s="8" t="str">
+        <x:v>一年分春夏秋冬四时</x:v>
+      </x:c>
+      <x:c r="H2080" s="8" t="str">
+        <x:v>一年分孟仲季十二个月</x:v>
+      </x:c>
+      <x:c r="I2080" s="8" t="str">
+        <x:v>一年分二十四节气</x:v>
+      </x:c>
+      <x:c r="J2080" s="8" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="K2080" s="8" t="str">
+        <x:v>商周以前一年只分春秋二时，“春秋”可代指一年，故古史书多以“春秋”为名。</x:v>
+      </x:c>
+      <x:c r="L2080" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2081">
+      <x:c r="A2081" s="3" t="n">
+        <x:v>2080</x:v>
+      </x:c>
+      <x:c r="B2081" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2081" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2081" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2081" s="3" t="str">
+        <x:v>古人将四季与五行、五方、五色相配，“夏”对应的方位与颜色是：</x:v>
+      </x:c>
+      <x:c r="F2081" s="8" t="str">
+        <x:v>南方、赤</x:v>
+      </x:c>
+      <x:c r="G2081" s="8" t="str">
+        <x:v>北方、黑</x:v>
+      </x:c>
+      <x:c r="H2081" s="8" t="str">
+        <x:v>东方、青</x:v>
+      </x:c>
+      <x:c r="I2081" s="8" t="str">
+        <x:v>西方、白</x:v>
+      </x:c>
+      <x:c r="J2081" s="8" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="K2081" s="8" t="str">
+        <x:v>“夏之神在南方，属丙丁火，色赤”，故夏配南方与赤色；春东方青、秋西方白、冬北方黑。</x:v>
+      </x:c>
+      <x:c r="L2081" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2082">
+      <x:c r="A2082" s="3" t="n">
+        <x:v>2081</x:v>
+      </x:c>
+      <x:c r="B2082" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2082" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2082" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2082" s="3" t="str">
+        <x:v>关于农历置月与四季，下列说法符合教材的是：</x:v>
+      </x:c>
+      <x:c r="F2082" s="8" t="str">
+        <x:v>农历以朔望月为月，平均长度约 29 日 12 时 4 分 3 秒</x:v>
+      </x:c>
+      <x:c r="G2082" s="8" t="str">
+        <x:v>大月 30 天小月 29 天且严格固定交替</x:v>
+      </x:c>
+      <x:c r="H2082" s="8" t="str">
+        <x:v>四季一律按中原平均气温均分九十天</x:v>
+      </x:c>
+      <x:c r="I2082" s="8" t="str">
+        <x:v>孟春、仲春、季春分别对应农历十月、十一月、十二月</x:v>
+      </x:c>
+      <x:c r="J2082" s="8" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="K2082" s="8" t="str">
+        <x:v>农历以月相盈亏为月，朔望月平均约 29 日 12 时 44 分；大小月不固定交替；孟春等对应正月、二月、三月。</x:v>
+      </x:c>
+      <x:c r="L2082" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2083">
+      <x:c r="A2083" s="3" t="n">
+        <x:v>2082</x:v>
+      </x:c>
+      <x:c r="B2083" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2083" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2083" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2083" s="3" t="str">
+        <x:v>汉代天文学所说的“五星”指五大行星，下列不属于“五星”的是：</x:v>
+      </x:c>
+      <x:c r="F2083" s="8" t="str">
+        <x:v>金星</x:v>
+      </x:c>
+      <x:c r="G2083" s="8" t="str">
+        <x:v>木星</x:v>
+      </x:c>
+      <x:c r="H2083" s="8" t="str">
+        <x:v>水星</x:v>
+      </x:c>
+      <x:c r="I2083" s="8" t="str">
+        <x:v>天王星</x:v>
+      </x:c>
+      <x:c r="J2083" s="8" t="str">
+        <x:v>D</x:v>
+      </x:c>
+      <x:c r="K2083" s="8" t="str">
+        <x:v>“五星”为太白（金星）、岁星（木星）、辰星（水星）、荧惑（火星）、镇星（土星），天王星为近代所发现。</x:v>
+      </x:c>
+      <x:c r="L2083" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2084">
+      <x:c r="A2084" s="3" t="n">
+        <x:v>2083</x:v>
+      </x:c>
+      <x:c r="B2084" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2084" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2084" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2084" s="3" t="str">
+        <x:v>星占语境中“五星出东方利中国”的“中国”指的是：</x:v>
+      </x:c>
+      <x:c r="F2084" s="8" t="str">
+        <x:v>全国范围</x:v>
+      </x:c>
+      <x:c r="G2084" s="8" t="str">
+        <x:v>黄河流域的中原地区</x:v>
+      </x:c>
+      <x:c r="H2084" s="8" t="str">
+        <x:v>华夏民族</x:v>
+      </x:c>
+      <x:c r="I2084" s="8" t="str">
+        <x:v>整个中国政权</x:v>
+      </x:c>
+      <x:c r="J2084" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2084" s="8" t="str">
+        <x:v>古星占中“中国”泛指黄河流域中原地区，其外为“西方”“夷狄”等。</x:v>
+      </x:c>
+      <x:c r="L2084" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2085">
+      <x:c r="A2085" s="3" t="n">
+        <x:v>2084</x:v>
+      </x:c>
+      <x:c r="B2085" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2085" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2085" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2085" s="3" t="str">
+        <x:v>关于“五星聚合”（五星连珠）的出现频率，下列说法正确的是：</x:v>
+      </x:c>
+      <x:c r="F2085" s="8" t="str">
+        <x:v>每隔几十年必然出现一次</x:v>
+      </x:c>
+      <x:c r="G2085" s="8" t="str">
+        <x:v>最近一次发生在 1921 年</x:v>
+      </x:c>
+      <x:c r="H2085" s="8" t="str">
+        <x:v>一般需要几十年乃至上百年才出现一次</x:v>
+      </x:c>
+      <x:c r="I2085" s="8" t="str">
+        <x:v>下一次聚合将在 2050 年前后</x:v>
+      </x:c>
+      <x:c r="J2085" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2085" s="8" t="str">
+        <x:v>五星聚合一般数十年至上百年一遇（如 1921 年，预计 2040 年前后再现），并非固定周期或必然事件。</x:v>
+      </x:c>
+      <x:c r="L2085" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2086">
+      <x:c r="A2086" s="3" t="n">
+        <x:v>2085</x:v>
+      </x:c>
+      <x:c r="B2086" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2086" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2086" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2086" s="3" t="str">
+        <x:v>阴阳合历需要“置闰”的根本原因是：</x:v>
+      </x:c>
+      <x:c r="F2086" s="8" t="str">
+        <x:v>朔望月周期与太阳年周期不能整除</x:v>
+      </x:c>
+      <x:c r="G2086" s="8" t="str">
+        <x:v>古人同时观察太阳与月亮</x:v>
+      </x:c>
+      <x:c r="H2086" s="8" t="str">
+        <x:v>阴历平年仅 354 天，少于太阳年</x:v>
+      </x:c>
+      <x:c r="I2086" s="8" t="str">
+        <x:v>置闰无定制，有时一年再闰</x:v>
+      </x:c>
+      <x:c r="J2086" s="8" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="K2086" s="8" t="str">
+        <x:v>十二个朔望月约 354 天，比太阳年约 365¼ 天少约 11 天，两种周期不能整除，故设闰月使历年接近太阳年。</x:v>
+      </x:c>
+      <x:c r="L2086" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2087">
+      <x:c r="A2087" s="3" t="n">
+        <x:v>2086</x:v>
+      </x:c>
+      <x:c r="B2087" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2087" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2087" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2087" s="3" t="str">
+        <x:v>古历中“岁”与“年”的区别是：</x:v>
+      </x:c>
+      <x:c r="F2087" s="8" t="str">
+        <x:v>“岁”自正月初一至次年正月初一，“年”自冬至至下一冬至</x:v>
+      </x:c>
+      <x:c r="G2087" s="8" t="str">
+        <x:v>“岁”自今年某节气至明年同一节气，“年”自今年正月初一至明年正月初一</x:v>
+      </x:c>
+      <x:c r="H2087" s="8" t="str">
+        <x:v>二者都指回归年，仅名称不同</x:v>
+      </x:c>
+      <x:c r="I2087" s="8" t="str">
+        <x:v>“岁”为阴历周期，“年”为阳历周期</x:v>
+      </x:c>
+      <x:c r="J2087" s="8" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="K2087" s="8" t="str">
+        <x:v>“岁”指从今年某一节气到明年同一节气（如冬至到冬至），“年”指从正月初一到次年正月初一。</x:v>
+      </x:c>
+      <x:c r="L2087" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2088">
+      <x:c r="A2088" s="3" t="n">
+        <x:v>2087</x:v>
+      </x:c>
+      <x:c r="B2088" s="3" t="str">
+        <x:v>中华文化题库</x:v>
+      </x:c>
+      <x:c r="C2088" s="3" t="str">
+        <x:v>中国文化史概要·教材命题（视觉识别）</x:v>
+      </x:c>
+      <x:c r="D2088" s="3" t="str">
+        <x:v>单选题</x:v>
+      </x:c>
+      <x:c r="E2088" s="3" t="str">
+        <x:v>汉初闰月置于九月之后称“后九月”，原因是：</x:v>
+      </x:c>
+      <x:c r="F2088" s="8" t="str">
+        <x:v>殷周以来闰月固定置于岁末</x:v>
+      </x:c>
+      <x:c r="G2088" s="8" t="str">
+        <x:v>春秋时有一年再闰的十四月现象</x:v>
+      </x:c>
+      <x:c r="H2088" s="8" t="str">
+        <x:v>沿袭秦制以十月为岁首、九月为岁终</x:v>
+      </x:c>
+      <x:c r="I2088" s="8" t="str">
+        <x:v>上古闰月均置于年中如闰三月闰六月</x:v>
+      </x:c>
+      <x:c r="J2088" s="8" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="K2088" s="8" t="str">
+        <x:v>汉初沿秦制以十月为岁首、九月为岁终，故闰月置于九月后称“后九月”。</x:v>
+      </x:c>
+      <x:c r="L2088" s="8" t="str">
+        <x:v>教材命题(视觉识别)</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R201b40cc09b541b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb898ebb4ff1440f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>